<commit_message>
23/03: Update de rama
</commit_message>
<xml_diff>
--- a/planificacion.xlsx
+++ b/planificacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Mis Carpetas\Especializacion\Big Data Aplicado\proyecto_big_data\EmKyu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FDC18F-327A-4BDE-9A5E-E3989D2FFC05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A94417-BA91-4198-8B4C-00C0545C1EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{C2B9D8F0-6321-49E0-921D-73330AFEBF0C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C2B9D8F0-6321-49E0-921D-73330AFEBF0C}"/>
   </bookViews>
   <sheets>
     <sheet name="PLANNING" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="27">
   <si>
     <t>FASE</t>
   </si>
@@ -221,13 +221,206 @@
     <t>Guardar desde Kafka en la DB Druid.
 Buena divisón de DB para sintéticos y reales.
 Configuración de hiperparámetros para un buen funcionamiento.</t>
+  </si>
+  <si>
+    <t>TAREAS</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">1) </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Scrapping </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>con actualización ventas de 4 monedas. ISAÍAS
+--Recurrente.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+2) </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Scrapping </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">apertura y cierre de mercado con 4 monedas. ADRIÁN
+--1 vez al día. SE PUEDE CALCULAR CON LA 1)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">3) </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Scrapping </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">con </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Order Book </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>en función de las 4 monedas</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ISAÍAS
+--Recurrente.</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">4) </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Scrapping </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Arbitraje entre 2 Brókers en función de las 4 monedas. ADRIÁN
+--Recurrente. SE PUEDE CALCULAR CON LA 1)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -261,6 +454,15 @@
     </font>
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -305,7 +507,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -325,6 +527,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -659,7 +865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39D5D314-C77B-4241-A15E-BE8F43F1B3F5}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
@@ -689,146 +895,157 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="11" t="s">
         <v>19</v>
       </c>
+      <c r="C3" s="11"/>
     </row>
     <row r="4" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="12" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:3" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C6" s="7">
         <v>46099</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" s="11" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="C7" s="11"/>
+    </row>
+    <row r="8" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C9" s="7">
         <v>46101</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" s="11" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="C10" s="11"/>
+    </row>
+    <row r="11" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+    <row r="12" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B12" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C12" s="7">
         <v>46106</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B13" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="10"/>
-    </row>
-    <row r="13" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="C13" s="10"/>
+    </row>
+    <row r="14" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>18</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>18</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B22" s="1" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>